<commit_message>
updated imaging preprocessing to accept long format and integrated imaging data from registry
</commit_message>
<xml_diff>
--- a/preprocessing/geneva_stroke_unit_preprocessing/variable_assembly/selected_variables_with_imaging.xlsx
+++ b/preprocessing/geneva_stroke_unit_preprocessing/variable_assembly/selected_variables_with_imaging.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jk1/stroke_research/OPSUM/preprocessing/geneva_stroke_unit_preprocessing/variable_assembly/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDD3E408-108C-9343-BD25-2034E13F391A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E517F4B7-9018-8745-8471-398CE639F430}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{4EF3017B-64DF-5142-A0B6-DCCDE5805A97}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="35840" windowHeight="21000" xr2:uid="{4EF3017B-64DF-5142-A0B6-DCCDE5805A97}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="88">
   <si>
     <t>Activite anti-Xa (DOAC)</t>
   </si>
@@ -287,13 +287,25 @@
   </si>
   <si>
     <t>phosphates</t>
+  </si>
+  <si>
+    <t>hypoperfusion_with_mismatch</t>
+  </si>
+  <si>
+    <t>hypoperfusion_without_mismatch</t>
+  </si>
+  <si>
+    <t>vascular_occlusion</t>
+  </si>
+  <si>
+    <t>vascular_stenosis_over_50p</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -316,6 +328,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF0F4A85"/>
+      <name val="Menlo"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -337,11 +355,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -656,7 +676,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E68269D3-7424-0349-8C48-DE37DFBA5500}">
-  <dimension ref="A1:D65"/>
+  <dimension ref="A1:E69"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -1037,9 +1057,31 @@
         <v>80</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>81</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
+        <v>84</v>
+      </c>
+      <c r="E66" s="4"/>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
+        <v>85</v>
+      </c>
+      <c r="E67" s="5"/>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
automate selection of parameters to normalize
</commit_message>
<xml_diff>
--- a/preprocessing/geneva_stroke_unit_preprocessing/variable_assembly/selected_variables_with_imaging.xlsx
+++ b/preprocessing/geneva_stroke_unit_preprocessing/variable_assembly/selected_variables_with_imaging.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jk1/stroke_research/OPSUM/preprocessing/geneva_stroke_unit_preprocessing/variable_assembly/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E517F4B7-9018-8745-8471-398CE639F430}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F12BD5CD-B135-7746-B5A2-8A7ABD01C7D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="35840" windowHeight="21000" xr2:uid="{4EF3017B-64DF-5142-A0B6-DCCDE5805A97}"/>
+    <workbookView xWindow="17920" yWindow="600" windowWidth="17920" windowHeight="21800" xr2:uid="{4EF3017B-64DF-5142-A0B6-DCCDE5805A97}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="94">
   <si>
     <t>Activite anti-Xa (DOAC)</t>
   </si>
@@ -268,21 +268,6 @@
     <t>G-Sga-pH(T), ABL</t>
   </si>
   <si>
-    <t>T10</t>
-  </si>
-  <si>
-    <t>T8</t>
-  </si>
-  <si>
-    <t>T6</t>
-  </si>
-  <si>
-    <t>T4</t>
-  </si>
-  <si>
-    <t>CBF</t>
-  </si>
-  <si>
     <t>neutrophiles-nb abs</t>
   </si>
   <si>
@@ -299,6 +284,39 @@
   </si>
   <si>
     <t>vascular_stenosis_over_50p</t>
+  </si>
+  <si>
+    <t>cbv_lt_34</t>
+  </si>
+  <si>
+    <t>cbv_lt_38</t>
+  </si>
+  <si>
+    <t>cbv_lt_42</t>
+  </si>
+  <si>
+    <t>tmax_gt_10</t>
+  </si>
+  <si>
+    <t>tmax_gt_8</t>
+  </si>
+  <si>
+    <t>tmax_gt_6</t>
+  </si>
+  <si>
+    <t>tmax_gt_4</t>
+  </si>
+  <si>
+    <t>cbf_lt_30</t>
+  </si>
+  <si>
+    <t>cbf_lt_34</t>
+  </si>
+  <si>
+    <t>cbf_lt_38</t>
+  </si>
+  <si>
+    <t>cbf_lt_20</t>
   </si>
 </sst>
 </file>
@@ -676,7 +694,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E68269D3-7424-0349-8C48-DE37DFBA5500}">
-  <dimension ref="A1:E69"/>
+  <dimension ref="A1:E75"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -976,112 +994,142 @@
         <v>53</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>78</v>
+      </c>
+      <c r="D60" s="3"/>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>79</v>
+      </c>
+      <c r="E61" s="4"/>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>80</v>
+      </c>
+      <c r="E62" s="5"/>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A60" t="s">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
         <v>83</v>
       </c>
-      <c r="D60" s="3"/>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A61" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A62" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A63" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A64" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A65" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>84</v>
       </c>
-      <c r="E66" s="4"/>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>85</v>
       </c>
-      <c r="E67" s="5"/>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>87</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A74" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A75" t="s">
+        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>